<commit_message>
Give Trichomonas vaginalis tissues that TISSUES has data for
Urethra has no rows in TISSUES and vagina only single-source HPA antibody
data, so no host protein passed the tissue filter and the parasite had no
predictions. Add uterine cervix, prostate and urinary tract, which it
also colonises: 216 predictions on 112 parasite proteins, no other
species affected.
</commit_message>
<xml_diff>
--- a/data/Parasites-db-Ida.xlsx
+++ b/data/Parasites-db-Ida.xlsx
@@ -2155,17 +2155,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>vagina, urethra</t>
+          <t>vagina, urethra, uterine cervix, prostate, urinary tract</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>BTO:0000243, BTO:0001426</t>
+          <t>BTO:0000243, BTO:0001426, BTO:0001421, BTO:0001129, BTO:0001244</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Urethra has no data in TISSUES and vagina only single-source HPA antibody data (25 proteins at cutoff 2.5), so on their own the parasite gets no predictions</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2405,7 +2410,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6313,6 +6318,70 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Trichomonas vaginalis</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>tissue</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>vagina, urethra</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>vagina, urethra, uterine cervix, prostate, urinary tract</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>cervix and prostate are colonised sites (cervicitis, prostatitis); urinary tract is the closest ancestor of urethra with TISSUES data. Urethra has no TISSUES rows at all and vagina only single-source HPA antibody data, so with the original two terms no host protein passed the tissue filter and the parasite had zero predictions</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Trichomonas vaginalis</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>BTO_id</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>BTO:0000243, BTO:0001426</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>BTO:0000243, BTO:0001426, BTO:0001421, BTO:0001129, BTO:0001244</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>biology</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>cervix and prostate are colonised sites (cervicitis, prostatitis); urinary tract is the closest ancestor of urethra with TISSUES data. Urethra has no TISSUES rows at all and vagina only single-source HPA antibody data, so with the original two terms no host protein passed the tissue filter and the parasite had zero predictions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Nippostrongylus brasiliensis as a rat and mouse parasite
Multicellular, extracellular nematode with a hookworm-like migration:
skin, blood, lung, small intestine. DeepLoc Accurate keeps 3,269 of its
22,636 proteins as secreted, giving 1,623 predicted PPIs (901 rat, 722
mouse) on 195 parasite proteins; no other species changes.
</commit_message>
<xml_diff>
--- a/data/Parasites-db-Ida.xlsx
+++ b/data/Parasites-db-Ida.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1306,11 +1306,11 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>6282</v>
+        <v>27835</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Onchocerca volvulus</t>
+          <t>Nippostrongylus brasiliensis</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1325,37 +1325,37 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Skin, eye</t>
+          <t>skin, blood, lung, small intestine</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000439</t>
+          <t>BTO:0001253, BTO:0000089, BTO:0000763, BTO:0000651</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Homo sapiens</t>
+          <t>Rattus norvegicus, Mus musculus</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Vector: blackfly(genusSimulium)</t>
+          <t>Natural parasite of rats and the standard mouse laboratory model of a hookworm-like life cycle: L3 penetrate the skin, reach the lungs through the blood within a day, are coughed up and swallowed, and mature in the jejunum, where adults are expelled around day 10.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>CDC, (Lustigman et al., 2018)</t>
+          <t>(Camberis et al., 2003), (Bouchery et al., 2017)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>147828</v>
+        <v>6282</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Opisthorchis felineus</t>
+          <t>Onchocerca volvulus</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1370,12 +1370,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Liver, bile duct, small intestine</t>
+          <t>Skin, eye</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0000122, BTO:0000651</t>
+          <t>BTO:0001253, BTO:0000439</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1383,19 +1383,24 @@
           <t>Homo sapiens</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Vector: blackfly(genusSimulium)</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>(Pakharukova &amp; Mordvinov, 2016)., CDC</t>
+          <t>CDC, (Lustigman et al., 2018)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>6198</v>
+        <v>147828</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Opisthorchis viverrini</t>
+          <t>Opisthorchis felineus</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1410,12 +1415,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Liver, bile duct</t>
+          <t>Liver, bile duct, small intestine</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0000122</t>
+          <t>BTO:0000759, BTO:0000122, BTO:0000651</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1425,37 +1430,37 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>(Sripa et al., 2025)</t>
+          <t>(Pakharukova &amp; Mordvinov, 2016)., CDC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>36329</v>
+        <v>6198</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Plasmodium falciparum</t>
+          <t>Opisthorchis viverrini</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Intracellular</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Skin, liver, blood, brain, spleen</t>
+          <t>Liver, bile duct</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000089, BTO:0000142, BTO:0001281</t>
+          <t>BTO:0000759, BTO:0000122</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1465,17 +1470,17 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>(Sripa et al., 2025)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>5851</v>
+        <v>36329</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Plasmodium knowlesi</t>
+          <t>Plasmodium falciparum</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1490,12 +1495,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Skin, liver, blood</t>
+          <t>Skin, liver, blood, brain, spleen</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000089</t>
+          <t>BTO:0001253, BTO:0000759, BTO:0000089, BTO:0000142, BTO:0001281</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1503,24 +1508,19 @@
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>macaques as natural host</t>
-        </is>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>(Singh &amp; Daneshvar, 2013), (White, 2008)</t>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>126793</v>
+        <v>5851</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Plasmodium vivax</t>
+          <t>Plasmodium knowlesi</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1548,49 +1548,49 @@
           <t>Homo sapiens</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>macaques as natural host</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>(Singh &amp; Daneshvar, 2013), (White, 2008)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>6185</v>
+        <v>126793</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Schistosoma haematobium</t>
+          <t>Plasmodium vivax</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Extracellular</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Skin, urinary bladder, rectum, liver, blood, lung</t>
+          <t>Skin, liver, blood</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0001418, BTO:0001158, BTO:0000759, BTO:0000089, BTO:0000763</t>
+          <t>BTO:0001253, BTO:0000759, BTO:0000089</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Intermediate hosts are snails of the genera Bulinus</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1601,11 +1601,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>6182</v>
+        <v>6185</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Schistosoma japonicum</t>
+          <t>Schistosoma haematobium</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1620,12 +1620,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Skin, liver, small intestine, lung, blood</t>
+          <t>Skin, urinary bladder, rectum, liver, blood, lung</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000763, BTO:0000089</t>
+          <t>BTO:0001253, BTO:0001418, BTO:0001158, BTO:0000759, BTO:0000089, BTO:0000763</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1635,22 +1635,22 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Intermediate hosts are snails of the genus Oncomelania</t>
+          <t>Intermediate hosts are snails of the genera Bulinus</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>CDC, (Zhou et al., 2009)</t>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>6183</v>
+        <v>6182</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Schistosoma mansoni</t>
+          <t>Schistosoma japonicum</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1665,12 +1665,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Skin, liver, intestine, spleen, lung, blood</t>
+          <t>Skin, liver, small intestine, lung, blood</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0001281, BTO:0000763, BTO:0000089</t>
+          <t>BTO:0001253, BTO:0000759, BTO:0000651, BTO:0000763, BTO:0000089</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1680,22 +1680,22 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Intermediate hosts are snails of the genus Biomphalaria spp</t>
+          <t>Intermediate hosts are snails of the genus Oncomelania</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>CDC, (Zhou et al., 2009)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>6248</v>
+        <v>6183</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Strongyloides stercoralis</t>
+          <t>Schistosoma mansoni</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1710,12 +1710,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>skin, lung, small intestine</t>
+          <t>Skin, liver, intestine, spleen, lung, blood</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
+          <t>BTO:0001253, BTO:0000759, BTO:0000648, BTO:0001281, BTO:0000763, BTO:0000089</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1723,19 +1723,24 @@
           <t>Homo sapiens</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Intermediate hosts are snails of the genus Biomphalaria spp</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>CDC, (Czeresnia &amp; Weiss, 2022)</t>
+          <t>CDC</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>60517</v>
+        <v>6248</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Taenia asiatica</t>
+          <t>Strongyloides stercoralis</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1750,12 +1755,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>small intestine</t>
+          <t>skin, lung, small intestine</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>BTO:0000651</t>
+          <t>BTO:0001253, BTO:0000763, BTO:0000651</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1763,24 +1768,19 @@
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>pigs as intermediate host</t>
-        </is>
-      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>(Parija, 2022)</t>
+          <t>CDC, (Czeresnia &amp; Weiss, 2022)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>6265</v>
+        <v>60517</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Toxocara canis</t>
+          <t>Taenia asiatica</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1795,12 +1795,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>liver, heart, lung, brain, muscle, eye</t>
+          <t>small intestine</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>BTO:0000759, BTO:0000562, BTO:0000763, BTO:0000142, BTO:0000887, BTO:0000439</t>
+          <t>BTO:0000651</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1810,42 +1810,42 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>humans are accidental hosts who become infected by ingesting infective eggs image or undercooked meat/viscera of infected paratenic hosts</t>
+          <t>pigs as intermediate host</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>CDC, (Schwartz et al., 2022)</t>
+          <t>(Parija, 2022)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>432359</v>
+        <v>6265</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Toxoplasma gondii</t>
+          <t>Toxocara canis</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Intracellular</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Blood, brain, eye, heart, muscle, placenta, lymph node</t>
+          <t>liver, heart, lung, brain, muscle, eye</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078, BTO:0000784</t>
+          <t>BTO:0000759, BTO:0000562, BTO:0000763, BTO:0000142, BTO:0000887, BTO:0000439</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1855,22 +1855,22 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>T. gondii can naturally infect a wide range of warm-blooded intermediate hosts, ranging from birds to humans to rodents.</t>
+          <t>humans are accidental hosts who become infected by ingesting infective eggs image or undercooked meat/viscera of infected paratenic hosts</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>CDC, (Kochanowsky &amp; Koshy, 2018)</t>
+          <t>CDC, (Schwartz et al., 2022)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>72359</v>
+        <v>432359</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Trachipleistophora hominis</t>
+          <t>Toxoplasma gondii</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1885,12 +1885,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Muscle, eye</t>
+          <t>Blood, brain, eye, heart, muscle, placenta, lymph node</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>BTO:0000887, BTO:0000439</t>
+          <t>BTO:0000089, BTO:0000142, BTO:0000439, BTO:0000562, BTO:0000887, BTO:0001078, BTO:0000784</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1900,27 +1900,27 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>natural host for T. hominis belongs to the hymenoptera.</t>
+          <t>T. gondii can naturally infect a wide range of warm-blooded intermediate hosts, ranging from birds to humans to rodents.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>CDC, (Watson et al., 2015)</t>
+          <t>CDC, (Kochanowsky &amp; Koshy, 2018)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>45882</v>
+        <v>72359</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Trichinella britovi</t>
+          <t>Trachipleistophora hominis</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Intestine, muscle, brain, heart, lung</t>
+          <t>Muscle, eye</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
+          <t>BTO:0000887, BTO:0000439</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1945,22 +1945,22 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Most of the Homo sapiens cases occurring globally are due to pork consumption, carnivores of Europe and western Asia (Wild boar, red fox, raccoon dog</t>
+          <t>natural host for T. hominis belongs to the hymenoptera.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>CDC, (Sharma et al., 2022)., (Pozio et al., 2009)</t>
+          <t>CDC, (Watson et al., 2015)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>6335</v>
+        <v>45882</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Trichinella nativa</t>
+          <t>Trichinella britovi</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1990,22 +1990,22 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>polar bears, American mink, Arctic fox, Asian badger, badger, black bears, Wolverine (Gulo gulo)</t>
+          <t>Most of the Homo sapiens cases occurring globally are due to pork consumption, carnivores of Europe and western Asia (Wild boar, red fox, raccoon dog</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>CDC, (Sharma et al., 2022), (Malone et al., 2025)</t>
+          <t>CDC, (Sharma et al., 2022)., (Pozio et al., 2009)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>6336</v>
+        <v>6335</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Trichinella nelsoni</t>
+          <t>Trichinella nativa</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2035,22 +2035,22 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Lion (Panthera leo), spotted hyena (Crocuta crocuta), leopard (Panthera pardus), cheetah (Actinonyx jubatus), bat-eared fox (Otocyon megalotis)</t>
+          <t>polar bears, American mink, Arctic fox, Asian badger, badger, black bears, Wolverine (Gulo gulo)</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>CDC, (Mukaratirwa et al., 2013)</t>
+          <t>CDC, (Sharma et al., 2022), (Malone et al., 2025)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>6337</v>
+        <v>6336</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Trichinella pseudospiralis</t>
+          <t>Trichinella nelsoni</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2075,27 +2075,27 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Homo sapiens, Sus scrofa</t>
+          <t>Homo sapiens</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>mammals and birds worldwide, mountain lion (Puma concolor), wolverine, wild boars and 8 avian species 3 species of Accipitridae; 1 species of Cathartidae; 1 species of Corvidae; 1 species of Tytonidae; 2 species of Strigidae</t>
+          <t>Lion (Panthera leo), spotted hyena (Crocuta crocuta), leopard (Panthera pardus), cheetah (Actinonyx jubatus), bat-eared fox (Otocyon megalotis)</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>(Pozio, 2016)</t>
+          <t>CDC, (Mukaratirwa et al., 2013)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>6334</v>
+        <v>6337</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Trichinella spiralis</t>
+          <t>Trichinella pseudospiralis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2110,12 +2110,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Intestine, brain, heart, muscle, lung</t>
+          <t>Intestine, muscle, brain, heart, lung</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>BTO:0000648, BTO:0000142, BTO:0000562, BTO:0000887, BTO:0000763</t>
+          <t>BTO:0000648, BTO:0000887, BTO:0000142, BTO:0000562, BTO:0000763</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2125,72 +2125,72 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>found worldwide in many carnivorous and omnivorous animals including humans, wild boars, Domestic pigs and brown rats (Rattus norvegicus)</t>
+          <t>mammals and birds worldwide, mountain lion (Puma concolor), wolverine, wild boars and 8 avian species 3 species of Accipitridae; 1 species of Cathartidae; 1 species of Corvidae; 1 species of Tytonidae; 2 species of Strigidae</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>CDC, (Sharma et al., 2022), (Pozio &amp; Gomez Morales, 2023), (Pozio et al., 2009)</t>
+          <t>(Pozio, 2016)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>5722</v>
+        <v>6334</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Trichomonas vaginalis</t>
+          <t>Trichinella spiralis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Extracellular</t>
+          <t>Intracellular</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>vagina, urethra, uterine cervix, prostate, urinary tract</t>
+          <t>Intestine, brain, heart, muscle, lung</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>BTO:0000243, BTO:0001426, BTO:0001421, BTO:0001129, BTO:0001244</t>
+          <t>BTO:0000648, BTO:0000142, BTO:0000562, BTO:0000887, BTO:0000763</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Homo sapiens</t>
+          <t>Homo sapiens, Sus scrofa</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Urethra has no data in TISSUES and vagina only single-source HPA antibody data (25 proteins at cutoff 2.5), so on their own the parasite gets no predictions</t>
+          <t>found worldwide in many carnivorous and omnivorous animals including humans, wild boars, Domestic pigs and brown rats (Rattus norvegicus)</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>CDC, (Kissinger, 2015)</t>
+          <t>CDC, (Sharma et al., 2022), (Pozio &amp; Gomez Morales, 2023), (Pozio et al., 2009)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>36087</v>
+        <v>5722</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Trichuris trichiura</t>
+          <t>Trichomonas vaginalis</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Multicellular</t>
+          <t>Unicellular</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2200,12 +2200,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>colon</t>
+          <t>vagina, urethra, uterine cervix, prostate, urinary tract</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>BTO:0000269</t>
+          <t>BTO:0000243, BTO:0001426, BTO:0001421, BTO:0001129, BTO:0001244</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2213,24 +2213,29 @@
           <t>Homo sapiens</t>
         </is>
       </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Urethra has no data in TISSUES and vagina only single-source HPA antibody data (25 proteins at cutoff 2.5), so on their own the parasite gets no predictions</t>
+        </is>
+      </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>CDC, (Izurieta et al., 2018)</t>
+          <t>CDC, (Kissinger, 2015)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>185431</v>
+        <v>36087</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Trypanosoma brucei</t>
+          <t>Trichuris trichiura</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Unicellular</t>
+          <t>Multicellular</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2240,12 +2245,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Skin, blood, brain, lymph node, spinal cord</t>
+          <t>colon</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000089, BTO:0000142, BTO:0000784, BTO:0001279</t>
+          <t>BTO:0000269</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2253,24 +2258,19 @@
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>T. brucei brucei is not infectious to Homo sapiens but can cause disease in cattle, goats, and sheep (i.e., nagana), andtherefore contributes to the societal impact of these diseases.</t>
-        </is>
-      </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>CDC, (Wang et al., 2008)</t>
+          <t>CDC, (Izurieta et al., 2018)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>353153</v>
+        <v>185431</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Trypanosoma cruzi</t>
+          <t>Trypanosoma brucei</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2280,17 +2280,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Intracellular</t>
+          <t>Extracellular</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Skin, heart, colon, muscle, blood, eye</t>
+          <t>Skin, blood, brain, lymph node, spinal cord</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>BTO:0001253, BTO:0000562, BTO:0000269, BTO:0000887, BTO:0000089, BTO:0000439</t>
+          <t>BTO:0001253, BTO:0000089, BTO:0000142, BTO:0000784, BTO:0001279</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2300,22 +2300,22 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>humans, armadillos, opossums, raccoons, woodrats, some other rodents, and domestic dogs.</t>
+          <t>T. brucei brucei is not infectious to Homo sapiens but can cause disease in cattle, goats, and sheep (i.e., nagana), andtherefore contributes to the societal impact of these diseases.</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>CDC</t>
+          <t>CDC, (Wang et al., 2008)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>993615</v>
+        <v>353153</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Vittaforma corneae</t>
+          <t>Trypanosoma cruzi</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2330,12 +2330,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>eye</t>
+          <t>Skin, heart, colon, muscle, blood, eye</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>BTO:0000439</t>
+          <t>BTO:0001253, BTO:0000562, BTO:0000269, BTO:0000887, BTO:0000089, BTO:0000439</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>No animal reservoir has been identified for Vittaforma cornea</t>
+          <t>humans, armadillos, opossums, raccoons, woodrats, some other rodents, and domestic dogs.</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2356,44 +2356,89 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
+        <v>993615</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Vittaforma corneae</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Unicellular</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Intracellular</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>eye</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>BTO:0000439</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Homo sapiens</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>No animal reservoir has been identified for Vittaforma cornea</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>CDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
         <v>6293</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Wuchereria bancrofti</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Multicellular</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Extracellular</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>blood, lymph node, lymph vessel</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>BTO:0000089, BTO:0000784, BTO:0000752</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>Transmitted by many different mosquito some genera include: Aedes spp., Anopheles spp., Culex spp., Mansonia spp., and Coquillettida juxtamansonia.</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>CDC, (Small et al., 2019)</t>
         </is>
@@ -2410,7 +2455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6382,6 +6427,38 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Nippostrongylus brasiliensis</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>(row)</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>(absent)</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Nippostrongylus brasiliensis</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>structure</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>added: rat-infecting nematode present in STRING v12 and EggNOG 6; multicellular, extracellular, skin/blood/lung/small intestine along the hookworm-like migration, hosts rat and mouse</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Record Leishmania braziliensis in human instead of rat
L. braziliensis is the principal agent of human mucocutaneous
leishmaniasis, and the tissues already recorded for it (skin, nose,
mouth, macrophage, blood) are the human presentation. Rat had no
standing for it and contributed nothing either: rat TISSUES carries no
annotation for any of those five tissues, so every rat protein was
dropped at the tissue filter.

Human adds 769 predictions, alongside mouse's 895. Regenerates
predictions.parquet and filter_stages.parquet, and updates the host
column and the changes log in Parasites-db-Ida.xlsx.
</commit_message>
<xml_diff>
--- a/data/Parasites-db-Ida.xlsx
+++ b/data/Parasites-db-Ida.xlsx
@@ -1135,7 +1135,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Rattus norvegicus, Mus musculus</t>
+          <t>Homo sapiens, Mus musculus</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2455,7 +2455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6459,6 +6459,38 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Leishmania braziliensis</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Rattus norvegicus, Mus musculus</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Homo sapiens, Mus musculus</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>the principal agent of human mucocutaneous leishmaniasis, and the recorded tissues (skin, nose, mouth, macrophage, blood) are the human presentation. Rattus norvegicus dropped: natural infection is reported in R. rattus and sylvatic rodents rather than the brown rat, and rat TISSUES carries no annotation for any of these five tissues, so it contributed no predictions</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>